<commit_message>
cambios finales, manuales y videos
</commit_message>
<xml_diff>
--- a/public/docs/base_docentes.xlsx
+++ b/public/docs/base_docentes.xlsx
@@ -1,60 +1,202 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nacho\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nacho\Desktop\front-gh\public\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED258F02-9B64-4867-85FF-D3F8AADC3108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{39CC5EA4-D163-4BF3-9A1A-0B65C0860581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{53973313-65D3-40DB-BDC3-E2B38B81610A}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="1"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
-  <si>
-    <t>Nombre</t>
-  </si>
-  <si>
-    <t>Contrato</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+  <si>
+    <t>Nombre del docente</t>
+  </si>
+  <si>
+    <t>Tipo de contrato</t>
+  </si>
+  <si>
+    <t>Carlos Valenzuela</t>
+  </si>
+  <si>
+    <t>Full-time</t>
+  </si>
+  <si>
+    <t>Patricia Olivares</t>
+  </si>
+  <si>
+    <t>Part-time</t>
+  </si>
+  <si>
+    <t>Mauricio Gaete</t>
+  </si>
+  <si>
+    <t>Loreto Espinoza</t>
+  </si>
+  <si>
+    <t>Hugo Silva</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
+  <fonts count="14">
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFCC0000"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF808080"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF006600"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color theme="1"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF0000EE"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF996600"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Liberation Sans"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <u/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Liberation Sans"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF808080"/>
+        <bgColor rgb="FF808080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDDDDD"/>
+        <bgColor rgb="FFDDDDDD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCCCC"/>
+        <bgColor rgb="FFFFCCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCC0000"/>
+        <bgColor rgb="FFCC0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCFFCC"/>
+        <bgColor rgb="FFCCFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -62,15 +204,68 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="20">
+    <cellStyle name="Accent" xfId="1" xr:uid="{6E226559-5651-4B0C-B0ED-304A4B3BF85F}"/>
+    <cellStyle name="Accent 1" xfId="2" xr:uid="{DB14DEBA-E0C7-45C1-A018-36B17BC471B3}"/>
+    <cellStyle name="Accent 2" xfId="3" xr:uid="{402968DC-633F-4736-A6B2-41C8F6EFA650}"/>
+    <cellStyle name="Accent 3" xfId="4" xr:uid="{FA3B4E8E-9DAE-43CF-8114-9211BED3D667}"/>
+    <cellStyle name="Bad" xfId="5" xr:uid="{53164F31-5707-4FFA-9118-F52978CB2DEF}"/>
+    <cellStyle name="Default" xfId="6" xr:uid="{96668123-D3C5-4B4F-9E2B-44666845280E}"/>
+    <cellStyle name="Error" xfId="7" xr:uid="{73E3C992-A583-4CBA-9A23-1B63D78EF55D}"/>
+    <cellStyle name="Footnote" xfId="8" xr:uid="{F893EA68-6962-4B01-8610-04E0317FD441}"/>
+    <cellStyle name="Good" xfId="9" xr:uid="{3C88BA95-3755-4F1D-8501-B6CF28FF3666}"/>
+    <cellStyle name="Heading" xfId="10" xr:uid="{4EE5692A-BC1E-45E4-9DF3-F46EB2D645FB}"/>
+    <cellStyle name="Heading 1" xfId="11" xr:uid="{FE54874E-D6D8-4725-8CA6-8FE6082D9BAC}"/>
+    <cellStyle name="Heading 2" xfId="12" xr:uid="{A0FA5FAF-C235-4E0B-B6DA-2E1205BAC35F}"/>
+    <cellStyle name="Hyperlink" xfId="13" xr:uid="{75024F17-97E6-493B-8C23-0FCE4235E5CF}"/>
+    <cellStyle name="Neutral" xfId="14" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
+    <cellStyle name="Note" xfId="15" xr:uid="{D863EA3D-6DAC-49D4-A6F9-F32C1270CD95}"/>
+    <cellStyle name="Result" xfId="16" xr:uid="{5332E2BE-2A25-485C-92B7-7763B7DE5089}"/>
+    <cellStyle name="Status" xfId="17" xr:uid="{51360401-6EB4-4D53-B7DF-FF856AE3C92D}"/>
+    <cellStyle name="Text" xfId="18" xr:uid="{0DB94C70-5534-4959-BCB6-BB2481B03073}"/>
+    <cellStyle name="Warning" xfId="19" xr:uid="{B7C662E2-6C93-4F96-A7E8-61FC9AEB6845}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -86,7 +281,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -96,42 +291,42 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic Light"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
@@ -161,12 +356,29 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
@@ -196,6 +408,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -257,13 +486,6 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -272,6 +494,13 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -336,22 +565,46 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A63DAA4D-581E-4C1E-8EB8-82D3AFCD6267}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.2"/>
+  <cols>
+    <col min="1" max="1" width="31.109375" customWidth="1"/>
+    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -359,7 +612,51 @@
         <v>1</v>
       </c>
     </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0" right="0" top="0.39370000000000011" bottom="0.39370000000000011" header="0" footer="0"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;A</oddHeader>
+    <oddFooter>&amp;CPage &amp;P</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>